<commit_message>
fix the problem of missing the end annotation data
</commit_message>
<xml_diff>
--- a/Analysed/Consolidated_Summary.xlsx
+++ b/Analysed/Consolidated_Summary.xlsx
@@ -533,52 +533,52 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2.5745</v>
+        <v>2.5787</v>
       </c>
       <c r="D2" t="n">
-        <v>1.1145</v>
+        <v>1.1092</v>
       </c>
       <c r="E2" t="n">
-        <v>2.9036</v>
+        <v>2.9084</v>
       </c>
       <c r="F2" t="n">
         <v>0.0672</v>
       </c>
       <c r="G2" t="n">
-        <v>3.3681</v>
+        <v>3.3624</v>
       </c>
       <c r="H2" t="n">
-        <v>2.3699</v>
+        <v>2.3759</v>
       </c>
       <c r="I2" t="n">
-        <v>3.5838</v>
+        <v>3.5806</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3984</v>
+        <v>0.4014</v>
       </c>
       <c r="K2" t="n">
-        <v>1.9921</v>
+        <v>1.9977</v>
       </c>
       <c r="L2" t="n">
-        <v>1.354</v>
+        <v>1.3673</v>
       </c>
       <c r="M2" t="n">
-        <v>2.4101</v>
+        <v>2.4136</v>
       </c>
       <c r="N2" t="n">
-        <v>0.4349</v>
+        <v>0.4345</v>
       </c>
       <c r="O2" t="n">
-        <v>4.6251</v>
+        <v>4.6252</v>
       </c>
       <c r="P2" t="n">
-        <v>2.0976</v>
+        <v>2.0981</v>
       </c>
       <c r="Q2" t="n">
-        <v>4.757</v>
+        <v>4.7572</v>
       </c>
       <c r="R2" t="n">
-        <v>0.7711</v>
+        <v>0.7707000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -593,28 +593,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2.9313</v>
+        <v>2.9494</v>
       </c>
       <c r="D3" t="n">
-        <v>2.7245</v>
+        <v>2.7351</v>
       </c>
       <c r="E3" t="n">
-        <v>3.4278</v>
+        <v>3.4459</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8185</v>
+        <v>0.8168</v>
       </c>
       <c r="G3" t="n">
-        <v>1.4791</v>
+        <v>1.4857</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2128</v>
+        <v>0.2226</v>
       </c>
       <c r="I3" t="n">
-        <v>1.7942</v>
+        <v>1.7999</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2848</v>
+        <v>0.2874</v>
       </c>
       <c r="K3" t="n">
         <v>1.2521</v>
@@ -653,16 +653,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2.9548</v>
+        <v>2.9517</v>
       </c>
       <c r="D4" t="n">
-        <v>3.2467</v>
+        <v>3.2497</v>
       </c>
       <c r="E4" t="n">
-        <v>3.3962</v>
+        <v>3.3935</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4748</v>
+        <v>0.4808</v>
       </c>
       <c r="G4" t="n">
         <v>0.678</v>
@@ -677,28 +677,28 @@
         <v>0.3459</v>
       </c>
       <c r="K4" t="n">
-        <v>1.1326</v>
+        <v>1.1261</v>
       </c>
       <c r="L4" t="n">
-        <v>2.0461</v>
+        <v>2.0493</v>
       </c>
       <c r="M4" t="n">
-        <v>1.27</v>
+        <v>1.2652</v>
       </c>
       <c r="N4" t="n">
-        <v>0.6036</v>
+        <v>0.6089</v>
       </c>
       <c r="O4" t="n">
-        <v>3.6725</v>
+        <v>3.6842</v>
       </c>
       <c r="P4" t="n">
-        <v>2.3012</v>
+        <v>2.3164</v>
       </c>
       <c r="Q4" t="n">
-        <v>4.0018</v>
+        <v>4.0126</v>
       </c>
       <c r="R4" t="n">
-        <v>0.7074</v>
+        <v>0.7089</v>
       </c>
     </row>
     <row r="5">
@@ -725,16 +725,16 @@
         <v>0.2847</v>
       </c>
       <c r="G5" t="n">
-        <v>12.5837</v>
+        <v>12.5727</v>
       </c>
       <c r="H5" t="n">
-        <v>6.4853</v>
+        <v>6.4726</v>
       </c>
       <c r="I5" t="n">
-        <v>13.23</v>
+        <v>13.2192</v>
       </c>
       <c r="J5" t="n">
-        <v>0.193</v>
+        <v>0.1951</v>
       </c>
       <c r="K5" t="n">
         <v>7.93</v>
@@ -773,52 +773,52 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>20.13</v>
+        <v>19.8362</v>
       </c>
       <c r="D6" t="n">
-        <v>6.7946</v>
+        <v>7.2353</v>
       </c>
       <c r="E6" t="n">
-        <v>20.3153</v>
+        <v>20.0689</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4823</v>
+        <v>0.463</v>
       </c>
       <c r="G6" t="n">
-        <v>16.6752</v>
+        <v>16.9717</v>
       </c>
       <c r="H6" t="n">
-        <v>1.5222</v>
+        <v>1.771</v>
       </c>
       <c r="I6" t="n">
-        <v>16.7947</v>
+        <v>17.099</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4421</v>
+        <v>0.4785</v>
       </c>
       <c r="K6" t="n">
-        <v>8.569800000000001</v>
+        <v>8.564500000000001</v>
       </c>
       <c r="L6" t="n">
-        <v>15.1006</v>
+        <v>15.29</v>
       </c>
       <c r="M6" t="n">
-        <v>8.6853</v>
+        <v>8.693199999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>0.5114</v>
+        <v>0.4998</v>
       </c>
       <c r="O6" t="n">
-        <v>1.6884</v>
+        <v>1.8734</v>
       </c>
       <c r="P6" t="n">
-        <v>0.622</v>
+        <v>0.8327</v>
       </c>
       <c r="Q6" t="n">
-        <v>2.1731</v>
+        <v>2.354</v>
       </c>
       <c r="R6" t="n">
-        <v>0.5109</v>
+        <v>0.5062</v>
       </c>
     </row>
     <row r="7">
@@ -833,52 +833,52 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>19.3934</v>
+        <v>19.3095</v>
       </c>
       <c r="D7" t="n">
-        <v>6.8231</v>
+        <v>6.9271</v>
       </c>
       <c r="E7" t="n">
-        <v>20.6621</v>
+        <v>20.6085</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4949</v>
+        <v>0.495</v>
       </c>
       <c r="G7" t="n">
-        <v>16.3331</v>
+        <v>16.3286</v>
       </c>
       <c r="H7" t="n">
-        <v>4.728</v>
+        <v>4.7169</v>
       </c>
       <c r="I7" t="n">
-        <v>16.3633</v>
+        <v>16.3588</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5242</v>
+        <v>0.5274</v>
       </c>
       <c r="K7" t="n">
-        <v>7.712</v>
+        <v>7.7191</v>
       </c>
       <c r="L7" t="n">
-        <v>14.6217</v>
+        <v>14.6189</v>
       </c>
       <c r="M7" t="n">
-        <v>7.8907</v>
+        <v>7.898</v>
       </c>
       <c r="N7" t="n">
-        <v>0.1915</v>
+        <v>0.197</v>
       </c>
       <c r="O7" t="n">
-        <v>1.0759</v>
+        <v>1.0744</v>
       </c>
       <c r="P7" t="n">
-        <v>0.2545</v>
+        <v>0.2527</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.3756</v>
+        <v>1.3746</v>
       </c>
       <c r="R7" t="n">
-        <v>0.3681</v>
+        <v>0.3691</v>
       </c>
     </row>
     <row r="8">
@@ -893,52 +893,52 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>25.9017</v>
+        <v>26.0424</v>
       </c>
       <c r="D8" t="n">
-        <v>8.3855</v>
+        <v>8.368499999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>29.8864</v>
+        <v>30.014</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1529</v>
+        <v>0.1487</v>
       </c>
       <c r="G8" t="n">
-        <v>21.6055</v>
+        <v>21.1366</v>
       </c>
       <c r="H8" t="n">
-        <v>12.1754</v>
+        <v>10.8921</v>
       </c>
       <c r="I8" t="n">
-        <v>24.0309</v>
+        <v>23.7025</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1348</v>
+        <v>0.1672</v>
       </c>
       <c r="K8" t="n">
-        <v>7.5763</v>
+        <v>7.7584</v>
       </c>
       <c r="L8" t="n">
-        <v>5.0923</v>
+        <v>5.3374</v>
       </c>
       <c r="M8" t="n">
-        <v>9.3596</v>
+        <v>9.5617</v>
       </c>
       <c r="N8" t="n">
-        <v>0.3911</v>
+        <v>0.3864</v>
       </c>
       <c r="O8" t="n">
-        <v>2.2522</v>
+        <v>2.1863</v>
       </c>
       <c r="P8" t="n">
-        <v>0.7943</v>
+        <v>0.7109</v>
       </c>
       <c r="Q8" t="n">
-        <v>2.7078</v>
+        <v>2.6488</v>
       </c>
       <c r="R8" t="n">
-        <v>0.7988</v>
+        <v>0.7748</v>
       </c>
     </row>
     <row r="9">
@@ -953,52 +953,52 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>28.3343</v>
+        <v>28.3608</v>
       </c>
       <c r="D9" t="n">
-        <v>10.3706</v>
+        <v>10.3564</v>
       </c>
       <c r="E9" t="n">
-        <v>30.5867</v>
+        <v>30.6165</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2559</v>
+        <v>0.2575</v>
       </c>
       <c r="G9" t="n">
-        <v>26.2183</v>
+        <v>26.2595</v>
       </c>
       <c r="H9" t="n">
-        <v>5.4672</v>
+        <v>5.5451</v>
       </c>
       <c r="I9" t="n">
-        <v>27.868</v>
+        <v>27.9116</v>
       </c>
       <c r="J9" t="n">
-        <v>0.3495</v>
+        <v>0.3494</v>
       </c>
       <c r="K9" t="n">
-        <v>23.1365</v>
+        <v>23.1472</v>
       </c>
       <c r="L9" t="n">
-        <v>20.0167</v>
+        <v>20.27</v>
       </c>
       <c r="M9" t="n">
-        <v>24.8016</v>
+        <v>24.8745</v>
       </c>
       <c r="N9" t="n">
-        <v>0.543</v>
+        <v>0.5249</v>
       </c>
       <c r="O9" t="n">
-        <v>2.6613</v>
+        <v>2.6598</v>
       </c>
       <c r="P9" t="n">
-        <v>1.3564</v>
+        <v>1.3462</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.1771</v>
+        <v>3.1784</v>
       </c>
       <c r="R9" t="n">
-        <v>0.7851</v>
+        <v>0.779</v>
       </c>
     </row>
     <row r="10">
@@ -1013,52 +1013,52 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>23.0295</v>
+        <v>22.7562</v>
       </c>
       <c r="D10" t="n">
-        <v>8.499700000000001</v>
+        <v>6.4634</v>
       </c>
       <c r="E10" t="n">
-        <v>24.9284</v>
+        <v>24.4275</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2606</v>
+        <v>0.2396</v>
       </c>
       <c r="G10" t="n">
-        <v>20.0609</v>
+        <v>20.1879</v>
       </c>
       <c r="H10" t="n">
-        <v>4.227</v>
+        <v>3.2086</v>
       </c>
       <c r="I10" t="n">
-        <v>20.8223</v>
+        <v>20.9132</v>
       </c>
       <c r="J10" t="n">
-        <v>0.3156</v>
+        <v>0.2847</v>
       </c>
       <c r="K10" t="n">
-        <v>19.472</v>
+        <v>16.9568</v>
       </c>
       <c r="L10" t="n">
-        <v>20.9921</v>
+        <v>17.1382</v>
       </c>
       <c r="M10" t="n">
-        <v>20.2435</v>
+        <v>17.7511</v>
       </c>
       <c r="N10" t="n">
-        <v>0.3525</v>
+        <v>0.3653</v>
       </c>
       <c r="O10" t="n">
-        <v>4.4417</v>
+        <v>4.4646</v>
       </c>
       <c r="P10" t="n">
-        <v>1.6019</v>
+        <v>1.2123</v>
       </c>
       <c r="Q10" t="n">
-        <v>5.5214</v>
+        <v>5.5238</v>
       </c>
       <c r="R10" t="n">
-        <v>0.3411</v>
+        <v>0.358</v>
       </c>
     </row>
   </sheetData>
@@ -1179,34 +1179,34 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.7896</v>
+        <v>1.783</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7798</v>
+        <v>0.7846</v>
       </c>
       <c r="E2" t="n">
-        <v>2.0625</v>
+        <v>2.0585</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2038</v>
+        <v>0.2081</v>
       </c>
       <c r="G2" t="n">
-        <v>2.1217</v>
+        <v>2.1229</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8552999999999999</v>
+        <v>0.8585</v>
       </c>
       <c r="I2" t="n">
-        <v>2.3964</v>
+        <v>2.3972</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2463</v>
+        <v>0.2475</v>
       </c>
       <c r="K2" t="n">
-        <v>1.5103</v>
+        <v>1.5106</v>
       </c>
       <c r="L2" t="n">
-        <v>0.3751</v>
+        <v>0.3748</v>
       </c>
       <c r="M2" t="n">
         <v>1.8839</v>
@@ -1215,16 +1215,16 @@
         <v>0.4301</v>
       </c>
       <c r="O2" t="n">
-        <v>4.0424</v>
+        <v>4.0426</v>
       </c>
       <c r="P2" t="n">
-        <v>2.3305</v>
+        <v>2.3309</v>
       </c>
       <c r="Q2" t="n">
-        <v>4.1603</v>
+        <v>4.1606</v>
       </c>
       <c r="R2" t="n">
-        <v>0.727</v>
+        <v>0.7266</v>
       </c>
     </row>
     <row r="3">
@@ -1239,28 +1239,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.4008</v>
+        <v>1.3967</v>
       </c>
       <c r="D3" t="n">
-        <v>1.4924</v>
+        <v>1.4871</v>
       </c>
       <c r="E3" t="n">
-        <v>1.6628</v>
+        <v>1.6594</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6139</v>
+        <v>0.6105</v>
       </c>
       <c r="G3" t="n">
-        <v>1.4575</v>
+        <v>1.463</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2549</v>
+        <v>0.2582</v>
       </c>
       <c r="I3" t="n">
-        <v>1.7763</v>
+        <v>1.7815</v>
       </c>
       <c r="J3" t="n">
-        <v>0.3461</v>
+        <v>0.3486</v>
       </c>
       <c r="K3" t="n">
         <v>1.5833</v>
@@ -1299,52 +1299,52 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.4889</v>
+        <v>1.508</v>
       </c>
       <c r="D4" t="n">
-        <v>1.4647</v>
+        <v>1.486</v>
       </c>
       <c r="E4" t="n">
-        <v>1.7539</v>
+        <v>1.7768</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3005</v>
+        <v>0.2989</v>
       </c>
       <c r="G4" t="n">
-        <v>1.0609</v>
+        <v>1.0607</v>
       </c>
       <c r="H4" t="n">
-        <v>1.2301</v>
+        <v>1.2397</v>
       </c>
       <c r="I4" t="n">
-        <v>1.2161</v>
+        <v>1.2168</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3493</v>
+        <v>0.3558</v>
       </c>
       <c r="K4" t="n">
-        <v>0.4195</v>
+        <v>0.4181</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1063</v>
+        <v>0.1122</v>
       </c>
       <c r="M4" t="n">
-        <v>0.6133999999999999</v>
+        <v>0.6115</v>
       </c>
       <c r="N4" t="n">
-        <v>0.6343</v>
+        <v>0.6325</v>
       </c>
       <c r="O4" t="n">
-        <v>1.6822</v>
+        <v>1.6831</v>
       </c>
       <c r="P4" t="n">
-        <v>2.3435</v>
+        <v>2.343</v>
       </c>
       <c r="Q4" t="n">
-        <v>1.9733</v>
+        <v>1.9741</v>
       </c>
       <c r="R4" t="n">
-        <v>0.7362</v>
+        <v>0.737</v>
       </c>
     </row>
     <row r="5">
@@ -1371,16 +1371,16 @@
         <v>0.3566</v>
       </c>
       <c r="G5" t="n">
-        <v>14.1132</v>
+        <v>14.1021</v>
       </c>
       <c r="H5" t="n">
-        <v>5.6129</v>
+        <v>5.6033</v>
       </c>
       <c r="I5" t="n">
-        <v>14.3245</v>
+        <v>14.3137</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3199</v>
+        <v>0.322</v>
       </c>
       <c r="K5" t="n">
         <v>2.2474</v>
@@ -1419,52 +1419,52 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>30.0701</v>
+        <v>30.3556</v>
       </c>
       <c r="D6" t="n">
-        <v>9.9641</v>
+        <v>10.3112</v>
       </c>
       <c r="E6" t="n">
-        <v>30.138</v>
+        <v>30.4278</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4474</v>
+        <v>0.4805</v>
       </c>
       <c r="G6" t="n">
-        <v>21.0901</v>
+        <v>21.3891</v>
       </c>
       <c r="H6" t="n">
-        <v>11.3919</v>
+        <v>11.1929</v>
       </c>
       <c r="I6" t="n">
-        <v>21.1708</v>
+        <v>21.477</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4736</v>
+        <v>0.5053</v>
       </c>
       <c r="K6" t="n">
-        <v>8.3208</v>
+        <v>8.1059</v>
       </c>
       <c r="L6" t="n">
-        <v>15.0746</v>
+        <v>15.1672</v>
       </c>
       <c r="M6" t="n">
-        <v>8.592599999999999</v>
+        <v>8.454499999999999</v>
       </c>
       <c r="N6" t="n">
-        <v>0.4459</v>
+        <v>0.4715</v>
       </c>
       <c r="O6" t="n">
-        <v>2.1441</v>
+        <v>2.352</v>
       </c>
       <c r="P6" t="n">
-        <v>0.4332</v>
+        <v>0.3907</v>
       </c>
       <c r="Q6" t="n">
-        <v>2.7615</v>
+        <v>2.962</v>
       </c>
       <c r="R6" t="n">
-        <v>0.4658</v>
+        <v>0.4831</v>
       </c>
     </row>
     <row r="7">
@@ -1479,52 +1479,52 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>21.7634</v>
+        <v>21.7057</v>
       </c>
       <c r="D7" t="n">
-        <v>3.828</v>
+        <v>3.8056</v>
       </c>
       <c r="E7" t="n">
-        <v>21.967</v>
+        <v>21.9228</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4909</v>
+        <v>0.4914</v>
       </c>
       <c r="G7" t="n">
-        <v>14.9272</v>
+        <v>14.9226</v>
       </c>
       <c r="H7" t="n">
-        <v>1.6196</v>
+        <v>1.615</v>
       </c>
       <c r="I7" t="n">
-        <v>14.9589</v>
+        <v>14.9545</v>
       </c>
       <c r="J7" t="n">
-        <v>0.515</v>
+        <v>0.5181</v>
       </c>
       <c r="K7" t="n">
-        <v>13.2899</v>
+        <v>13.2927</v>
       </c>
       <c r="L7" t="n">
-        <v>18.8059</v>
+        <v>18.8035</v>
       </c>
       <c r="M7" t="n">
-        <v>13.431</v>
+        <v>13.4339</v>
       </c>
       <c r="N7" t="n">
-        <v>0.4918</v>
+        <v>0.4939</v>
       </c>
       <c r="O7" t="n">
-        <v>1.2747</v>
+        <v>1.2743</v>
       </c>
       <c r="P7" t="n">
-        <v>0.4165</v>
+        <v>0.417</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.5767</v>
+        <v>1.5762</v>
       </c>
       <c r="R7" t="n">
-        <v>0.415</v>
+        <v>0.416</v>
       </c>
     </row>
     <row r="8">
@@ -1539,52 +1539,52 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>44.4532</v>
+        <v>44.7435</v>
       </c>
       <c r="D8" t="n">
-        <v>28.2156</v>
+        <v>29.3701</v>
       </c>
       <c r="E8" t="n">
-        <v>50.8898</v>
+        <v>51.0304</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1822</v>
+        <v>0.2059</v>
       </c>
       <c r="G8" t="n">
-        <v>25.4987</v>
+        <v>26.1025</v>
       </c>
       <c r="H8" t="n">
-        <v>11.4172</v>
+        <v>11.5988</v>
       </c>
       <c r="I8" t="n">
-        <v>29.3734</v>
+        <v>29.9557</v>
       </c>
       <c r="J8" t="n">
-        <v>0.07389999999999999</v>
+        <v>0.08260000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>15.3938</v>
+        <v>15.5</v>
       </c>
       <c r="L8" t="n">
-        <v>17.4709</v>
+        <v>17.4345</v>
       </c>
       <c r="M8" t="n">
-        <v>16.5831</v>
+        <v>16.6708</v>
       </c>
       <c r="N8" t="n">
-        <v>0.4309</v>
+        <v>0.4036</v>
       </c>
       <c r="O8" t="n">
-        <v>2.1072</v>
+        <v>2.1098</v>
       </c>
       <c r="P8" t="n">
-        <v>1.2451</v>
+        <v>1.2292</v>
       </c>
       <c r="Q8" t="n">
-        <v>2.5009</v>
+        <v>2.488</v>
       </c>
       <c r="R8" t="n">
-        <v>0.7786999999999999</v>
+        <v>0.7546</v>
       </c>
     </row>
     <row r="9">
@@ -1599,52 +1599,52 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>20.6511</v>
+        <v>20.6776</v>
       </c>
       <c r="D9" t="n">
-        <v>5.3029</v>
+        <v>5.2958</v>
       </c>
       <c r="E9" t="n">
-        <v>22.38</v>
+        <v>22.4099</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4697</v>
+        <v>0.4713</v>
       </c>
       <c r="G9" t="n">
-        <v>21.9198</v>
+        <v>21.9463</v>
       </c>
       <c r="H9" t="n">
-        <v>7.1873</v>
+        <v>7.2079</v>
       </c>
       <c r="I9" t="n">
-        <v>23.1189</v>
+        <v>23.1485</v>
       </c>
       <c r="J9" t="n">
-        <v>0.472</v>
+        <v>0.4736</v>
       </c>
       <c r="K9" t="n">
-        <v>14.6968</v>
+        <v>14.917</v>
       </c>
       <c r="L9" t="n">
-        <v>17.0044</v>
+        <v>17.3306</v>
       </c>
       <c r="M9" t="n">
-        <v>16.3395</v>
+        <v>16.5774</v>
       </c>
       <c r="N9" t="n">
-        <v>0.502</v>
+        <v>0.4947</v>
       </c>
       <c r="O9" t="n">
-        <v>2.3685</v>
+        <v>2.3654</v>
       </c>
       <c r="P9" t="n">
-        <v>1.3018</v>
+        <v>1.2901</v>
       </c>
       <c r="Q9" t="n">
-        <v>2.8311</v>
+        <v>2.8325</v>
       </c>
       <c r="R9" t="n">
-        <v>0.7634</v>
+        <v>0.7573</v>
       </c>
     </row>
     <row r="10">
@@ -1659,52 +1659,52 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>16.9828</v>
+        <v>21.5423</v>
       </c>
       <c r="D10" t="n">
-        <v>4.7065</v>
+        <v>12.2585</v>
       </c>
       <c r="E10" t="n">
-        <v>17.9492</v>
+        <v>22.3912</v>
       </c>
       <c r="F10" t="n">
-        <v>0.3028</v>
+        <v>0.2748</v>
       </c>
       <c r="G10" t="n">
-        <v>21.0337</v>
+        <v>19.3803</v>
       </c>
       <c r="H10" t="n">
-        <v>1.918</v>
+        <v>4.4791</v>
       </c>
       <c r="I10" t="n">
-        <v>22.3071</v>
+        <v>20.7527</v>
       </c>
       <c r="J10" t="n">
-        <v>0.3001</v>
+        <v>0.3251</v>
       </c>
       <c r="K10" t="n">
-        <v>15.2607</v>
+        <v>20.7376</v>
       </c>
       <c r="L10" t="n">
-        <v>26.0047</v>
+        <v>23.2391</v>
       </c>
       <c r="M10" t="n">
-        <v>16.3533</v>
+        <v>21.6652</v>
       </c>
       <c r="N10" t="n">
-        <v>0.2654</v>
+        <v>0.2378</v>
       </c>
       <c r="O10" t="n">
-        <v>4.4397</v>
+        <v>4.488</v>
       </c>
       <c r="P10" t="n">
-        <v>1.1807</v>
+        <v>0.9113</v>
       </c>
       <c r="Q10" t="n">
-        <v>5.5735</v>
+        <v>5.6232</v>
       </c>
       <c r="R10" t="n">
-        <v>0.3471</v>
+        <v>0.3421</v>
       </c>
     </row>
   </sheetData>

</xml_diff>